<commit_message>
Fix text truncation in workbooks (sector/name/industry columns)
Sector (sic_description) was hard-sliced at 32 chars and columns capped at 42
wide, so values like "Retail-Auto Dealers & Gasoline Stations" showed cut off.
Raised descriptive-text slices (name/sector/industry/company) to 40-60 chars
across universe/style/people renders, and lifted the autosize width cap 42->62
(measuring up to 80). Comma-list and short-flag columns left as-is. Full sector
and company names now display.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzLWQfQoCmwwwE2QTFQZro
</commit_message>
<xml_diff>
--- a/people_monitor.xlsx
+++ b/people_monitor.xlsx
@@ -528,7 +528,7 @@
   <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -892,7 +892,7 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="9.5" customWidth="1" min="3" max="3"/>
     <col width="11.5" customWidth="1" min="4" max="4"/>
@@ -1009,9 +1009,9 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="19.5" customWidth="1" min="2" max="2"/>
-    <col width="26.5" customWidth="1" min="3" max="3"/>
+    <col width="29.5" customWidth="1" min="3" max="3"/>
     <col width="8.5" customWidth="1" min="4" max="4"/>
     <col width="11.5" customWidth="1" min="5" max="5"/>
     <col width="10.5" customWidth="1" min="6" max="6"/>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>ABB (Distributors/Wholes</t>
+          <t>ABB (Distributors/Wholesale</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Orascom Development Hold</t>
+          <t>Orascom Development Holding</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Silicon Motion Technolog</t>
+          <t>Silicon Motion Technology</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -1806,12 +1806,12 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="8.5" customWidth="1" min="2" max="2"/>
     <col width="13.5" customWidth="1" min="3" max="3"/>
     <col width="12.5" customWidth="1" min="4" max="4"/>
-    <col width="32.5" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="50.5" customWidth="1" min="5" max="5"/>
+    <col width="42.5" customWidth="1" min="6" max="6"/>
     <col width="11.5" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1882,7 +1882,7 @@
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Aston Martin Lagonda Global Ho</t>
+          <t>Aston Martin Lagonda Global Holdings</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Billionaire/Oligarch Vehicles,</t>
+          <t>Billionaire/Oligarch Vehicles,Titans &amp; Concentra</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -1999,9 +1999,9 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="13.5" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="46.5" customWidth="1" min="3" max="3"/>
     <col width="30.5" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -2129,7 +2129,7 @@
   <dimension ref="A1:F204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="30.5" customWidth="1" min="2" max="2"/>
     <col width="22.5" customWidth="1" min="3" max="3"/>
     <col width="24.5" customWidth="1" min="4" max="4"/>
@@ -8615,7 +8615,7 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="36.5" customWidth="1" min="2" max="2"/>
     <col width="10.5" customWidth="1" min="3" max="3"/>
     <col width="10.5" customWidth="1" min="4" max="4"/>

</xml_diff>